<commit_message>
chore: Atualização das simulações
</commit_message>
<xml_diff>
--- a/docs/simulacoes/Cenario_Sustentabilidade.xlsx
+++ b/docs/simulacoes/Cenario_Sustentabilidade.xlsx
@@ -5,10 +5,10 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="5"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="1" activeTab="5"/>
   </bookViews>
   <sheets>
-    <sheet name="Parametros" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="Parametros" sheetId="1" state="hidden" r:id="rId3"/>
     <sheet name="AHP_Dimensoes" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Pesos_Indicadores" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="Normalizacao" sheetId="4" state="visible" r:id="rId6"/>
@@ -1101,7 +1101,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="43">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1158,7 +1158,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="12" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1238,7 +1238,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="11" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1263,10 +1263,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="171" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="12" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -24218,14 +24214,14 @@
         <f aca="false">IF(OR(NOT(ISNUMBER(B7)),NOT(ISNUMBER(C7))),"",C7-B7)</f>
         <v>0</v>
       </c>
-      <c r="E7" s="41" t="str">
+      <c r="E7" s="14" t="str">
         <f aca="false">IF(D7="","",IF(ABS(D7)&lt;=Parametros!$B$49,"OK","DIVERGE"))</f>
         <v>OK</v>
       </c>
       <c r="F7" s="6" t="s">
         <v>248</v>
       </c>
-      <c r="G7" s="42" t="n">
+      <c r="G7" s="41" t="n">
         <v>0.818181818181818</v>
       </c>
     </row>
@@ -24244,14 +24240,14 @@
         <f aca="false">IF(OR(NOT(ISNUMBER(B8)),NOT(ISNUMBER(C8))),"",C8-B8)</f>
         <v>0</v>
       </c>
-      <c r="E8" s="41" t="str">
+      <c r="E8" s="14" t="str">
         <f aca="false">IF(D8="","",IF(ABS(D8)&lt;=Parametros!$B$49,"OK","DIVERGE"))</f>
         <v>OK</v>
       </c>
       <c r="F8" s="6" t="s">
         <v>248</v>
       </c>
-      <c r="G8" s="42" t="n">
+      <c r="G8" s="41" t="n">
         <v>0.0909090909090909</v>
       </c>
     </row>
@@ -24270,14 +24266,14 @@
         <f aca="false">IF(OR(NOT(ISNUMBER(B9)),NOT(ISNUMBER(C9))),"",C9-B9)</f>
         <v>0</v>
       </c>
-      <c r="E9" s="41" t="str">
+      <c r="E9" s="14" t="str">
         <f aca="false">IF(D9="","",IF(ABS(D9)&lt;=Parametros!$B$49,"OK","DIVERGE"))</f>
         <v>OK</v>
       </c>
       <c r="F9" s="6" t="s">
         <v>248</v>
       </c>
-      <c r="G9" s="42" t="n">
+      <c r="G9" s="41" t="n">
         <v>0.0909090909090909</v>
       </c>
     </row>
@@ -24296,14 +24292,14 @@
         <f aca="false">IF(OR(NOT(ISNUMBER(B10)),NOT(ISNUMBER(C10))),"",C10-B10)</f>
         <v>0</v>
       </c>
-      <c r="E10" s="41" t="str">
+      <c r="E10" s="14" t="str">
         <f aca="false">IF(D10="","",IF(ABS(D10)&lt;=Parametros!$B$49,"OK","DIVERGE"))</f>
         <v>OK</v>
       </c>
       <c r="F10" s="6" t="s">
         <v>252</v>
       </c>
-      <c r="G10" s="42" t="n">
+      <c r="G10" s="41" t="n">
         <v>3</v>
       </c>
     </row>
@@ -24322,14 +24318,14 @@
         <f aca="false">IF(OR(NOT(ISNUMBER(B11)),NOT(ISNUMBER(C11))),"",C11-B11)</f>
         <v>0</v>
       </c>
-      <c r="E11" s="41" t="str">
+      <c r="E11" s="14" t="str">
         <f aca="false">IF(D11="","",IF(ABS(D11)&lt;=Parametros!$B$49,"OK","DIVERGE"))</f>
         <v>OK</v>
       </c>
       <c r="F11" s="6" t="s">
         <v>252</v>
       </c>
-      <c r="G11" s="42" t="n">
+      <c r="G11" s="41" t="n">
         <v>0</v>
       </c>
     </row>
@@ -24348,14 +24344,14 @@
         <f aca="false">IF(OR(NOT(ISNUMBER(B12)),NOT(ISNUMBER(C12))),"",C12-B12)</f>
         <v>0</v>
       </c>
-      <c r="E12" s="41" t="str">
+      <c r="E12" s="14" t="str">
         <f aca="false">IF(D12="","",IF(ABS(D12)&lt;=Parametros!$B$49,"OK","DIVERGE"))</f>
         <v>OK</v>
       </c>
       <c r="F12" s="6" t="s">
         <v>255</v>
       </c>
-      <c r="G12" s="42" t="n">
+      <c r="G12" s="41" t="n">
         <v>0.58</v>
       </c>
     </row>
@@ -24374,14 +24370,14 @@
         <f aca="false">IF(OR(NOT(ISNUMBER(B13)),NOT(ISNUMBER(C13))),"",C13-B13)</f>
         <v>0</v>
       </c>
-      <c r="E13" s="41" t="str">
+      <c r="E13" s="14" t="str">
         <f aca="false">IF(D13="","",IF(ABS(D13)&lt;=Parametros!$B$49,"OK","DIVERGE"))</f>
         <v>OK</v>
       </c>
       <c r="F13" s="6" t="s">
         <v>252</v>
       </c>
-      <c r="G13" s="42" t="n">
+      <c r="G13" s="41" t="n">
         <v>0</v>
       </c>
     </row>
@@ -24400,14 +24396,14 @@
         <f aca="false">IF(OR(NOT(ISNUMBER(B14)),NOT(ISNUMBER(C14))),"",C14-B14)</f>
         <v>0</v>
       </c>
-      <c r="E14" s="41" t="str">
+      <c r="E14" s="14" t="str">
         <f aca="false">IF(D14="","",IF(ABS(D14)&lt;=Parametros!$B$49,"OK","DIVERGE"))</f>
         <v>OK</v>
       </c>
       <c r="F14" s="6" t="s">
         <v>258</v>
       </c>
-      <c r="G14" s="42" t="n">
+      <c r="G14" s="41" t="n">
         <v>5</v>
       </c>
     </row>
@@ -24426,14 +24422,14 @@
         <f aca="false">IF(OR(NOT(ISNUMBER(B15)),NOT(ISNUMBER(C15))),"",C15-B15)</f>
         <v>0</v>
       </c>
-      <c r="E15" s="41" t="str">
+      <c r="E15" s="14" t="str">
         <f aca="false">IF(D15="","",IF(ABS(D15)&lt;=Parametros!$B$49,"OK","DIVERGE"))</f>
         <v>OK</v>
       </c>
       <c r="F15" s="6" t="s">
         <v>258</v>
       </c>
-      <c r="G15" s="42" t="n">
+      <c r="G15" s="41" t="n">
         <v>0.384615384615385</v>
       </c>
     </row>
@@ -24452,14 +24448,14 @@
         <f aca="false">IF(OR(NOT(ISNUMBER(B16)),NOT(ISNUMBER(C16))),"",C16-B16)</f>
         <v>0</v>
       </c>
-      <c r="E16" s="41" t="str">
+      <c r="E16" s="14" t="str">
         <f aca="false">IF(D16="","",IF(ABS(D16)&lt;=Parametros!$B$49,"OK","DIVERGE"))</f>
         <v>OK</v>
       </c>
       <c r="F16" s="6" t="s">
         <v>260</v>
       </c>
-      <c r="G16" s="42" t="n">
+      <c r="G16" s="41" t="n">
         <v>1</v>
       </c>
     </row>
@@ -24478,14 +24474,14 @@
         <f aca="false">IF(OR(NOT(ISNUMBER(B17)),NOT(ISNUMBER(C17))),"",C17-B17)</f>
         <v>2.85714285674921E-007</v>
       </c>
-      <c r="E17" s="41" t="str">
+      <c r="E17" s="14" t="str">
         <f aca="false">IF(D17="","",IF(ABS(D17)&lt;=Parametros!$B$49,"OK","DIVERGE"))</f>
         <v>OK</v>
       </c>
       <c r="F17" s="6" t="s">
         <v>262</v>
       </c>
-      <c r="G17" s="42" t="n">
+      <c r="G17" s="41" t="n">
         <v>0.910506</v>
       </c>
     </row>
@@ -24504,14 +24500,14 @@
         <f aca="false">IF(OR(NOT(ISNUMBER(B18)),NOT(ISNUMBER(C18))),"",C18-B18)</f>
         <v>-4.2857142858177E-007</v>
       </c>
-      <c r="E18" s="41" t="str">
+      <c r="E18" s="14" t="str">
         <f aca="false">IF(D18="","",IF(ABS(D18)&lt;=Parametros!$B$49,"OK","DIVERGE"))</f>
         <v>OK</v>
       </c>
       <c r="F18" s="6" t="s">
         <v>262</v>
       </c>
-      <c r="G18" s="42" t="n">
+      <c r="G18" s="41" t="n">
         <v>0.05114</v>
       </c>
     </row>
@@ -24530,14 +24526,14 @@
         <f aca="false">IF(OR(NOT(ISNUMBER(B19)),NOT(ISNUMBER(C19))),"",C19-B19)</f>
         <v>1.42857142851338E-007</v>
       </c>
-      <c r="E19" s="41" t="str">
+      <c r="E19" s="14" t="str">
         <f aca="false">IF(D19="","",IF(ABS(D19)&lt;=Parametros!$B$49,"OK","DIVERGE"))</f>
         <v>OK</v>
       </c>
       <c r="F19" s="6" t="s">
         <v>262</v>
       </c>
-      <c r="G19" s="42" t="n">
+      <c r="G19" s="41" t="n">
         <v>0.038355</v>
       </c>
     </row>
@@ -24556,14 +24552,14 @@
         <f aca="false">IF(OR(NOT(ISNUMBER(B20)),NOT(ISNUMBER(C20))),"",C20-B20)</f>
         <v>5.99656039268481E-008</v>
       </c>
-      <c r="E20" s="41" t="str">
+      <c r="E20" s="14" t="str">
         <f aca="false">IF(D20="","",IF(ABS(D20)&lt;=Parametros!$B$49,"OK","DIVERGE"))</f>
         <v>OK</v>
       </c>
       <c r="F20" s="6" t="s">
         <v>266</v>
       </c>
-      <c r="G20" s="42" t="n">
+      <c r="G20" s="41" t="n">
         <v>0.872233</v>
       </c>
     </row>
@@ -24582,14 +24578,14 @@
         <f aca="false">IF(OR(NOT(ISNUMBER(B21)),NOT(ISNUMBER(C21))),"",C21-B21)</f>
         <v>-4.30461787659375E-007</v>
       </c>
-      <c r="E21" s="41" t="str">
+      <c r="E21" s="14" t="str">
         <f aca="false">IF(D21="","",IF(ABS(D21)&lt;=Parametros!$B$49,"OK","DIVERGE"))</f>
         <v>OK</v>
       </c>
       <c r="F21" s="6" t="s">
         <v>266</v>
       </c>
-      <c r="G21" s="42" t="n">
+      <c r="G21" s="41" t="n">
         <v>0.897806</v>
       </c>
     </row>
@@ -24608,14 +24604,14 @@
         <f aca="false">IF(OR(NOT(ISNUMBER(B22)),NOT(ISNUMBER(C22))),"",C22-B22)</f>
         <v>-4.37354294446912E-007</v>
       </c>
-      <c r="E22" s="41" t="str">
+      <c r="E22" s="14" t="str">
         <f aca="false">IF(D22="","",IF(ABS(D22)&lt;=Parametros!$B$49,"OK","DIVERGE"))</f>
         <v>OK</v>
       </c>
       <c r="F22" s="6" t="s">
         <v>266</v>
       </c>
-      <c r="G22" s="42" t="n">
+      <c r="G22" s="41" t="n">
         <v>0.815129</v>
       </c>
     </row>
@@ -24634,14 +24630,14 @@
         <f aca="false">IF(OR(NOT(ISNUMBER(B23)),NOT(ISNUMBER(C23))),"",C23-B23)</f>
         <v>-4.90427391641735E-007</v>
       </c>
-      <c r="E23" s="41" t="str">
+      <c r="E23" s="14" t="str">
         <f aca="false">IF(D23="","",IF(ABS(D23)&lt;=Parametros!$B$49,"OK","DIVERGE"))</f>
         <v>OK</v>
       </c>
       <c r="F23" s="6" t="s">
         <v>269</v>
       </c>
-      <c r="G23" s="42" t="n">
+      <c r="G23" s="41" t="n">
         <v>0.025573</v>
       </c>
     </row>
@@ -24660,14 +24656,14 @@
         <f aca="false">IF(OR(NOT(ISNUMBER(B24)),NOT(ISNUMBER(C24))),"",C24-B24)</f>
         <v>1.81818181816951E-005</v>
       </c>
-      <c r="E24" s="41" t="str">
+      <c r="E24" s="14" t="str">
         <f aca="false">IF(D24="","",IF(ABS(D24)&lt;=Parametros!$B$49,"OK","DIVERGE"))</f>
         <v>OK</v>
       </c>
       <c r="F24" s="6" t="s">
         <v>271</v>
       </c>
-      <c r="G24" s="42" t="n">
+      <c r="G24" s="41" t="n">
         <v>-0.5032</v>
       </c>
     </row>
@@ -24684,14 +24680,14 @@
         <f aca="false">IF(OR(NOT(ISNUMBER(B25)),NOT(ISNUMBER(C25))),"",C25-B25)</f>
         <v/>
       </c>
-      <c r="E25" s="41" t="str">
+      <c r="E25" s="14" t="str">
         <f aca="false">IF(D25="","",IF(ABS(D25)&lt;=Parametros!$B$49,"OK","DIVERGE"))</f>
         <v/>
       </c>
       <c r="F25" s="6" t="s">
         <v>271</v>
       </c>
-      <c r="G25" s="42"/>
+      <c r="G25" s="41"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="6" t="s">
@@ -24708,14 +24704,14 @@
         <f aca="false">IF(OR(NOT(ISNUMBER(B26)),NOT(ISNUMBER(C26))),"",C26-B26)</f>
         <v>-9.09090909084753E-006</v>
       </c>
-      <c r="E26" s="41" t="str">
+      <c r="E26" s="14" t="str">
         <f aca="false">IF(D26="","",IF(ABS(D26)&lt;=Parametros!$B$49,"OK","DIVERGE"))</f>
         <v>OK</v>
       </c>
       <c r="F26" s="6" t="s">
         <v>271</v>
       </c>
-      <c r="G26" s="42" t="n">
+      <c r="G26" s="41" t="n">
         <v>0.4041</v>
       </c>
     </row>
@@ -24751,14 +24747,14 @@
         <f aca="false">Pontuacao!B38</f>
         <v>Google Cloud</v>
       </c>
-      <c r="E29" s="41" t="str">
+      <c r="E29" s="14" t="str">
         <f aca="false">IF(TRIM(B29&amp;"")=TRIM(C29&amp;""),"OK","DIVERGE")</f>
         <v>OK</v>
       </c>
       <c r="F29" s="6" t="s">
         <v>269</v>
       </c>
-      <c r="G29" s="43" t="s">
+      <c r="G29" s="42" t="s">
         <v>201</v>
       </c>
     </row>
@@ -24773,14 +24769,14 @@
         <f aca="false">AHP_Dimensoes!B36</f>
         <v>CONSISTENTE</v>
       </c>
-      <c r="E30" s="41" t="str">
+      <c r="E30" s="14" t="str">
         <f aca="false">IF(TRIM(B30&amp;"")=TRIM(C30&amp;""),"OK","DIVERGE")</f>
         <v>OK</v>
       </c>
       <c r="F30" s="6" t="s">
         <v>252</v>
       </c>
-      <c r="G30" s="43" t="s">
+      <c r="G30" s="42" t="s">
         <v>277</v>
       </c>
     </row>
@@ -24795,14 +24791,14 @@
         <f aca="false">Pontuacao!B40</f>
         <v>não</v>
       </c>
-      <c r="E31" s="41" t="str">
+      <c r="E31" s="14" t="str">
         <f aca="false">IF(TRIM(B31&amp;"")=TRIM(C31&amp;""),"OK","DIVERGE")</f>
         <v>OK</v>
       </c>
       <c r="F31" s="6" t="s">
         <v>269</v>
       </c>
-      <c r="G31" s="43" t="s">
+      <c r="G31" s="42" t="s">
         <v>208</v>
       </c>
     </row>
@@ -24817,14 +24813,14 @@
         <f aca="false">Pontuacao!B41</f>
         <v>não</v>
       </c>
-      <c r="E32" s="41" t="str">
+      <c r="E32" s="14" t="str">
         <f aca="false">IF(TRIM(B32&amp;"")=TRIM(C32&amp;""),"OK","DIVERGE")</f>
         <v>OK</v>
       </c>
       <c r="F32" s="6" t="s">
         <v>269</v>
       </c>
-      <c r="G32" s="43" t="s">
+      <c r="G32" s="42" t="s">
         <v>208</v>
       </c>
     </row>
@@ -24839,14 +24835,14 @@
         <f aca="false">COUNTIF(Normalizacao!$AG$5:$AG$17,"non_discriminative")</f>
         <v>0</v>
       </c>
-      <c r="E33" s="41" t="str">
+      <c r="E33" s="14" t="str">
         <f aca="false">IF(TRIM(B33&amp;"")=TRIM(C33&amp;""),"OK","DIVERGE")</f>
         <v>OK</v>
       </c>
       <c r="F33" s="6" t="s">
         <v>280</v>
       </c>
-      <c r="G33" s="43" t="n">
+      <c r="G33" s="42" t="n">
         <v>6</v>
       </c>
     </row>
@@ -24861,14 +24857,14 @@
         <f aca="false">Sensibilidade!B13</f>
         <v>Sustentabilidade</v>
       </c>
-      <c r="E34" s="41" t="str">
+      <c r="E34" s="14" t="str">
         <f aca="false">IF(TRIM(B34&amp;"")=TRIM(C34&amp;""),"OK","DIVERGE")</f>
         <v>OK</v>
       </c>
       <c r="F34" s="6" t="s">
         <v>271</v>
       </c>
-      <c r="G34" s="43" t="s">
+      <c r="G34" s="42" t="s">
         <v>62</v>
       </c>
     </row>
@@ -24876,14 +24872,14 @@
       <c r="A36" s="6" t="s">
         <v>281</v>
       </c>
-      <c r="B36" s="41" t="str">
+      <c r="B36" s="14" t="str">
         <f aca="false">IF(COUNTIF(E7:E34,"DIVERGE")=0,"OK — a planilha reproduz o relatório","DIVERGE em "&amp;COUNTIF(E7:E34,"DIVERGE")&amp;" grandeza(s)")</f>
         <v>OK — a planilha reproduz o relatório</v>
       </c>
-      <c r="C36" s="41"/>
-      <c r="D36" s="41"/>
-      <c r="E36" s="41"/>
-      <c r="F36" s="41"/>
+      <c r="C36" s="14"/>
+      <c r="D36" s="14"/>
+      <c r="E36" s="14"/>
+      <c r="F36" s="14"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="8" t="s">

</xml_diff>